<commit_message>
Fixed the DCF model to 23 lines.
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kyle\Desktop\Coding\Investment Research\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Project-Magnolia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5C5417-4A48-42CD-82DC-E41088B98A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FD4980-F34F-4EF5-80EB-A86DE5B3D2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Company Name</t>
   </si>
@@ -80,6 +80,12 @@
   </si>
   <si>
     <t>SharesOut</t>
+  </si>
+  <si>
+    <t>NOW MARKET CAP</t>
+  </si>
+  <si>
+    <t>Years</t>
   </si>
 </sst>
 </file>
@@ -115,9 +121,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,10 +482,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C852AD-020B-43B6-920C-38E6A80F8FCC}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
       <c r="B1" t="s">
         <v>10</v>
       </c>
@@ -503,8 +513,11 @@
       <c r="J1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -532,8 +545,11 @@
       <c r="J2">
         <v>1104</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K2" s="2">
+        <v>109400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -562,7 +578,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -591,7 +607,7 @@
         <v>1494</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -620,7 +636,7 @@
         <v>1914</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
       </c>

</xml_diff>

<commit_message>
Added a DCF model for KNSL
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Project-Magnolia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FD4980-F34F-4EF5-80EB-A86DE5B3D2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE7BF7A-820A-4371-93D5-F7E0C35A0334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="HWM_financials" sheetId="2" r:id="rId2"/>
+    <sheet name="KNSL_financials" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Company Name</t>
   </si>
@@ -92,8 +93,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -121,10 +130,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,7 +555,7 @@
       <c r="J2">
         <v>1104</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2">
         <v>109400</v>
       </c>
     </row>
@@ -668,4 +678,112 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C19A9A9-560B-4709-8B61-64F10DA3F3E3}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="17.26953125" style="3"/>
+    <col min="3" max="4" width="17.26953125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="C2" s="2">
+        <v>407</v>
+      </c>
+      <c r="D2" s="2">
+        <v>6</v>
+      </c>
+      <c r="K2">
+        <v>8100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="2">
+        <v>558</v>
+      </c>
+      <c r="D3" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="C4" s="2">
+        <v>860</v>
+      </c>
+      <c r="D4" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="C5" s="2">
+        <v>976</v>
+      </c>
+      <c r="D5" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1044</v>
+      </c>
+      <c r="D6" s="2">
+        <v>54</v>
+      </c>
+      <c r="F6">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Made one master DCF program to read multiple companies off the Excel file
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Project-Magnolia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE7BF7A-820A-4371-93D5-F7E0C35A0334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0FF886-9620-4D37-8098-91B5B9644472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="HWM_financials" sheetId="2" r:id="rId2"/>
-    <sheet name="KNSL_financials" sheetId="3" r:id="rId3"/>
+    <sheet name="Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="CompanyTemplate" sheetId="5" r:id="rId2"/>
+    <sheet name="HWM" sheetId="2" r:id="rId3"/>
+    <sheet name="KNSL" sheetId="3" r:id="rId4"/>
+    <sheet name="FIX" sheetId="4" r:id="rId5"/>
+    <sheet name="MU" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
   <si>
     <t>Company Name</t>
   </si>
@@ -50,59 +53,45 @@
     <t>HWM</t>
   </si>
   <si>
-    <t>Market Cap (In Billions)</t>
-  </si>
-  <si>
     <t>Howmet</t>
   </si>
   <si>
     <t>Kinsale</t>
   </si>
   <si>
-    <t>Revenue</t>
-  </si>
-  <si>
-    <t>EBIT (OI)</t>
-  </si>
-  <si>
-    <t>Dep + Amo</t>
-  </si>
-  <si>
-    <t>Cash</t>
-  </si>
-  <si>
     <t>OperatingCashFlow</t>
   </si>
   <si>
     <t>CapEx</t>
   </si>
   <si>
-    <t>TotalDebt</t>
-  </si>
-  <si>
     <t>SharesOut</t>
   </si>
   <si>
-    <t>NOW MARKET CAP</t>
-  </si>
-  <si>
     <t>Years</t>
+  </si>
+  <si>
+    <t>MarketCap</t>
+  </si>
+  <si>
+    <t>FIX</t>
+  </si>
+  <si>
+    <t>Comfort Systems</t>
+  </si>
+  <si>
+    <t>MU</t>
+  </si>
+  <si>
+    <t>Micron Technology</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -133,8 +122,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -433,7 +422,7 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -447,13 +436,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1">
-        <v>109.4</v>
+      <c r="C2" s="3">
+        <v>109400</v>
       </c>
       <c r="D2" s="1">
         <v>1.83</v>
@@ -467,13 +456,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1">
-        <v>8.6999999999999993</v>
+      <c r="C3" s="3">
+        <v>8700</v>
       </c>
       <c r="D3" s="1">
         <v>13.21</v>
@@ -483,6 +472,28 @@
       </c>
       <c r="F3" s="1">
         <v>21.67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3">
+        <v>60900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3">
+        <v>833600</v>
       </c>
     </row>
   </sheetData>
@@ -491,188 +502,47 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C852AD-020B-43B6-920C-38E6A80F8FCC}">
-  <dimension ref="A1:K6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F6EFFA6-3D4E-40CB-9167-9611E0BB3DF4}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
       <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2021</v>
       </c>
-      <c r="B2">
-        <v>4972</v>
-      </c>
-      <c r="C2">
-        <v>449</v>
-      </c>
-      <c r="D2">
-        <v>199</v>
-      </c>
-      <c r="E2">
-        <v>4308</v>
-      </c>
-      <c r="F2">
-        <v>422</v>
-      </c>
-      <c r="H2">
-        <v>720</v>
-      </c>
-      <c r="I2">
-        <v>270</v>
-      </c>
-      <c r="J2">
-        <v>1104</v>
-      </c>
-      <c r="K2">
-        <v>109400</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3">
-        <v>5663</v>
-      </c>
-      <c r="C3">
-        <v>733</v>
-      </c>
-      <c r="D3">
-        <v>193</v>
-      </c>
-      <c r="E3">
-        <v>4245</v>
-      </c>
-      <c r="F3">
-        <v>412</v>
-      </c>
-      <c r="H3">
-        <v>791</v>
-      </c>
-      <c r="I3">
-        <v>265</v>
-      </c>
-      <c r="J3">
-        <v>1273</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4">
-        <v>6640</v>
-      </c>
-      <c r="C4">
-        <v>901</v>
-      </c>
-      <c r="D4">
-        <v>219</v>
-      </c>
-      <c r="E4">
-        <v>3597</v>
-      </c>
-      <c r="F4">
-        <v>410</v>
-      </c>
-      <c r="H4">
-        <v>610</v>
-      </c>
-      <c r="I4">
-        <v>272</v>
-      </c>
-      <c r="J4">
-        <v>1494</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5">
-        <v>7430</v>
-      </c>
-      <c r="C5">
-        <v>1298</v>
-      </c>
-      <c r="D5">
-        <v>321</v>
-      </c>
-      <c r="E5">
-        <v>3428</v>
-      </c>
-      <c r="F5">
-        <v>405</v>
-      </c>
-      <c r="H5">
-        <v>564</v>
-      </c>
-      <c r="I5">
-        <v>277</v>
-      </c>
-      <c r="J5">
-        <v>1914</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
-      </c>
-      <c r="B6">
-        <v>8252</v>
-      </c>
-      <c r="C6">
-        <v>1884</v>
-      </c>
-      <c r="D6">
-        <v>453</v>
-      </c>
-      <c r="E6">
-        <v>2980</v>
-      </c>
-      <c r="F6">
-        <v>402</v>
-      </c>
-      <c r="H6">
-        <v>742</v>
-      </c>
-      <c r="I6">
-        <v>283</v>
-      </c>
-      <c r="J6">
-        <v>2416</v>
       </c>
     </row>
   </sheetData>
@@ -681,104 +551,176 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C852AD-020B-43B6-920C-38E6A80F8FCC}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>449</v>
+      </c>
+      <c r="C2">
+        <v>199</v>
+      </c>
+      <c r="D2">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>733</v>
+      </c>
+      <c r="C3">
+        <v>193</v>
+      </c>
+      <c r="D3">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>901</v>
+      </c>
+      <c r="C4">
+        <v>219</v>
+      </c>
+      <c r="D4">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>1298</v>
+      </c>
+      <c r="C5">
+        <v>321</v>
+      </c>
+      <c r="D5">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>1884</v>
+      </c>
+      <c r="C6">
+        <v>453</v>
+      </c>
+      <c r="D6">
+        <v>402</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C19A9A9-560B-4709-8B61-64F10DA3F3E3}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.26953125" style="3"/>
-    <col min="3" max="4" width="17.26953125" style="2"/>
+    <col min="2" max="4" width="17.26953125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2021</v>
       </c>
+      <c r="B2" s="2">
+        <v>407</v>
+      </c>
       <c r="C2" s="2">
-        <v>407</v>
-      </c>
-      <c r="D2" s="2">
         <v>6</v>
       </c>
-      <c r="K2">
-        <v>8100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2022</v>
       </c>
+      <c r="B3" s="2">
+        <v>558</v>
+      </c>
       <c r="C3" s="2">
-        <v>558</v>
-      </c>
-      <c r="D3" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2023</v>
       </c>
+      <c r="B4" s="2">
+        <v>860</v>
+      </c>
       <c r="C4" s="2">
-        <v>860</v>
-      </c>
-      <c r="D4" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2024</v>
       </c>
+      <c r="B5" s="2">
+        <v>976</v>
+      </c>
       <c r="C5" s="2">
-        <v>976</v>
-      </c>
-      <c r="D5" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
       </c>
+      <c r="B6" s="2">
+        <v>1044</v>
+      </c>
       <c r="C6" s="2">
-        <v>1044</v>
+        <v>54</v>
       </c>
       <c r="D6" s="2">
-        <v>54</v>
-      </c>
-      <c r="F6">
         <v>23</v>
       </c>
     </row>
@@ -786,4 +728,171 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3935994C-2385-47E7-868B-A40B19ABC727}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="4" width="17.26953125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="2">
+        <v>180</v>
+      </c>
+      <c r="C2" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3" s="2">
+        <v>302</v>
+      </c>
+      <c r="C3" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="2">
+        <v>640</v>
+      </c>
+      <c r="C4" s="2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="2">
+        <v>849</v>
+      </c>
+      <c r="C5" s="2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1186</v>
+      </c>
+      <c r="C6" s="2">
+        <v>155</v>
+      </c>
+      <c r="D6" s="2">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B8453C4-6D6F-43DB-95E7-7C6D17636AFE}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>12468</v>
+      </c>
+      <c r="C2">
+        <v>10030</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>15181</v>
+      </c>
+      <c r="C3">
+        <v>12067</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>1559</v>
+      </c>
+      <c r="C4">
+        <v>7676</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>8507</v>
+      </c>
+      <c r="C5">
+        <v>8386</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>17525</v>
+      </c>
+      <c r="C6">
+        <v>15857</v>
+      </c>
+      <c r="D6">
+        <v>1122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added yFinance for automatic current stock prices and HTML and CSS for the website
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -8,17 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Project-Magnolia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0FF886-9620-4D37-8098-91B5B9644472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385F4F39-573D-4D0D-AF75-1AE6A5C0FEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
-    <sheet name="CompanyTemplate" sheetId="5" r:id="rId2"/>
+    <sheet name="ct" sheetId="5" r:id="rId2"/>
     <sheet name="HWM" sheetId="2" r:id="rId3"/>
     <sheet name="KNSL" sheetId="3" r:id="rId4"/>
     <sheet name="FIX" sheetId="4" r:id="rId5"/>
     <sheet name="MU" sheetId="6" r:id="rId6"/>
+    <sheet name="NBIS" sheetId="7" r:id="rId7"/>
+    <sheet name="MG" sheetId="9" r:id="rId8"/>
+    <sheet name="RGLD" sheetId="10" r:id="rId9"/>
+    <sheet name="MPWR" sheetId="13" r:id="rId10"/>
+    <sheet name="ABNB" sheetId="14" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
   <si>
     <t>Company Name</t>
   </si>
@@ -84,6 +89,36 @@
   </si>
   <si>
     <t>Micron Technology</t>
+  </si>
+  <si>
+    <t>NBIS</t>
+  </si>
+  <si>
+    <t>Nebius Group</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>Mistras Group</t>
+  </si>
+  <si>
+    <t>Royal Gold</t>
+  </si>
+  <si>
+    <t>RGLD</t>
+  </si>
+  <si>
+    <t>Monolithic Power Systems</t>
+  </si>
+  <si>
+    <t>MPWR</t>
+  </si>
+  <si>
+    <t>AirBNB</t>
+  </si>
+  <si>
+    <t>ABNB</t>
   </si>
 </sst>
 </file>
@@ -119,11 +154,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -441,7 +474,7 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2">
         <v>109400</v>
       </c>
       <c r="D2" s="1">
@@ -461,7 +494,7 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3">
         <v>8700</v>
       </c>
       <c r="D3" s="1">
@@ -481,7 +514,7 @@
       <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>60900</v>
       </c>
     </row>
@@ -492,8 +525,227 @@
       <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>833600</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6">
+        <v>47700</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>19150</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>109200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48FC485-1630-41C2-9709-BFBE7E263A58}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>320</v>
+      </c>
+      <c r="C2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>247</v>
+      </c>
+      <c r="C3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>638</v>
+      </c>
+      <c r="C4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>788</v>
+      </c>
+      <c r="C5">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>838</v>
+      </c>
+      <c r="C6">
+        <v>172</v>
+      </c>
+      <c r="D6">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{556EA6CB-4D7D-43A5-986F-1B79476B7661}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>2190</v>
+      </c>
+      <c r="C2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>3430</v>
+      </c>
+      <c r="C3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>3884</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>4518</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>4646</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>602</v>
       </c>
     </row>
   </sheetData>
@@ -648,21 +900,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C19A9A9-560B-4709-8B61-64F10DA3F3E3}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="4" width="17.26953125" style="2"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -670,10 +919,10 @@
       <c r="A2">
         <v>2021</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>407</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>6</v>
       </c>
     </row>
@@ -681,10 +930,10 @@
       <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>558</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3">
         <v>7</v>
       </c>
     </row>
@@ -692,10 +941,10 @@
       <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>860</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4">
         <v>7</v>
       </c>
     </row>
@@ -703,10 +952,10 @@
       <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>976</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>24</v>
       </c>
     </row>
@@ -714,13 +963,13 @@
       <c r="A6">
         <v>2025</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>1044</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>54</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>23</v>
       </c>
     </row>
@@ -734,21 +983,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3935994C-2385-47E7-868B-A40B19ABC727}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="4" width="17.26953125" style="2"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -756,10 +1002,10 @@
       <c r="A2">
         <v>2021</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>180</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>22</v>
       </c>
     </row>
@@ -767,10 +1013,10 @@
       <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>302</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3">
         <v>48</v>
       </c>
     </row>
@@ -778,10 +1024,10 @@
       <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>640</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4">
         <v>95</v>
       </c>
     </row>
@@ -789,10 +1035,10 @@
       <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>849</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>111</v>
       </c>
     </row>
@@ -800,13 +1046,13 @@
       <c r="A6">
         <v>2025</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>1186</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>155</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>35</v>
       </c>
     </row>
@@ -895,4 +1141,250 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44815C06-4B74-477E-90B9-68CA77F13F20}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>124</v>
+      </c>
+      <c r="C2">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>572</v>
+      </c>
+      <c r="C3">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>782</v>
+      </c>
+      <c r="C4">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>246</v>
+      </c>
+      <c r="C5">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>385</v>
+      </c>
+      <c r="C6">
+        <v>4066</v>
+      </c>
+      <c r="D6">
+        <v>253</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{211ECC06-B714-41A3-8304-4E9A77B12D43}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>42261</v>
+      </c>
+      <c r="C2">
+        <v>15396</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>26406</v>
+      </c>
+      <c r="C3">
+        <v>12591</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>26748</v>
+      </c>
+      <c r="C4">
+        <v>20854</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>50129</v>
+      </c>
+      <c r="C5">
+        <v>17092</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>32981</v>
+      </c>
+      <c r="C6">
+        <v>24674</v>
+      </c>
+      <c r="D6">
+        <v>31567</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03B05C2C-F23D-4154-B9E7-6674A908B62A}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>407</v>
+      </c>
+      <c r="C2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>417</v>
+      </c>
+      <c r="C3">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>416</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>530</v>
+      </c>
+      <c r="C5">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>705</v>
+      </c>
+      <c r="C6">
+        <v>1165</v>
+      </c>
+      <c r="D6">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
10: Housekeeping + more automations
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -8,22 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Project-Magnolia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385F4F39-573D-4D0D-AF75-1AE6A5C0FEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0C0EA0-45A5-490C-9962-9C776051C807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="834" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
-    <sheet name="ct" sheetId="5" r:id="rId2"/>
-    <sheet name="HWM" sheetId="2" r:id="rId3"/>
-    <sheet name="KNSL" sheetId="3" r:id="rId4"/>
-    <sheet name="FIX" sheetId="4" r:id="rId5"/>
-    <sheet name="MU" sheetId="6" r:id="rId6"/>
-    <sheet name="NBIS" sheetId="7" r:id="rId7"/>
-    <sheet name="MG" sheetId="9" r:id="rId8"/>
-    <sheet name="RGLD" sheetId="10" r:id="rId9"/>
-    <sheet name="MPWR" sheetId="13" r:id="rId10"/>
-    <sheet name="ABNB" sheetId="14" r:id="rId11"/>
+    <sheet name="Recs" sheetId="25" r:id="rId2"/>
+    <sheet name="ct" sheetId="5" r:id="rId3"/>
+    <sheet name="HWM" sheetId="2" r:id="rId4"/>
+    <sheet name="KNSL" sheetId="3" r:id="rId5"/>
+    <sheet name="FIX" sheetId="4" r:id="rId6"/>
+    <sheet name="MU" sheetId="6" r:id="rId7"/>
+    <sheet name="NBIS" sheetId="7" r:id="rId8"/>
+    <sheet name="MG" sheetId="9" r:id="rId9"/>
+    <sheet name="RGLD" sheetId="10" r:id="rId10"/>
+    <sheet name="MPWR" sheetId="13" r:id="rId11"/>
+    <sheet name="ABNB" sheetId="14" r:id="rId12"/>
+    <sheet name="B" sheetId="18" r:id="rId13"/>
+    <sheet name="MCEM" sheetId="19" r:id="rId14"/>
+    <sheet name="AGI" sheetId="20" r:id="rId15"/>
+    <sheet name="CRM" sheetId="21" r:id="rId16"/>
+    <sheet name="EXEL" sheetId="22" r:id="rId17"/>
+    <sheet name="KGC" sheetId="24" r:id="rId18"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="80">
   <si>
     <t>Company Name</t>
   </si>
@@ -119,6 +126,162 @@
   </si>
   <si>
     <t>ABNB</t>
+  </si>
+  <si>
+    <t>Barrick Mining</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>MCEM</t>
+  </si>
+  <si>
+    <t>Monarch Cement</t>
+  </si>
+  <si>
+    <t>AGI</t>
+  </si>
+  <si>
+    <t>CRM</t>
+  </si>
+  <si>
+    <t>Salesforce</t>
+  </si>
+  <si>
+    <t>Exelixis</t>
+  </si>
+  <si>
+    <t>EXEL</t>
+  </si>
+  <si>
+    <t>Kinross Gold</t>
+  </si>
+  <si>
+    <t>KGC</t>
+  </si>
+  <si>
+    <t>MEDP</t>
+  </si>
+  <si>
+    <t>NFLX</t>
+  </si>
+  <si>
+    <t>TSLA</t>
+  </si>
+  <si>
+    <t>HD</t>
+  </si>
+  <si>
+    <t>CMG</t>
+  </si>
+  <si>
+    <t>GOOGL</t>
+  </si>
+  <si>
+    <t>LLY</t>
+  </si>
+  <si>
+    <t>CAT</t>
+  </si>
+  <si>
+    <t>COST</t>
+  </si>
+  <si>
+    <t>HMC</t>
+  </si>
+  <si>
+    <t>MSFT</t>
+  </si>
+  <si>
+    <t>Alphabet</t>
+  </si>
+  <si>
+    <t>AMZN</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>META</t>
+  </si>
+  <si>
+    <t>Meta Platforms</t>
+  </si>
+  <si>
+    <t>AAPL</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>NVDA</t>
+  </si>
+  <si>
+    <t>NVIDIA</t>
+  </si>
+  <si>
+    <t>AVGO</t>
+  </si>
+  <si>
+    <t>Broadcom</t>
+  </si>
+  <si>
+    <t>JPM</t>
+  </si>
+  <si>
+    <t>JPMorgan Chase</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Visa</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>Mastercard</t>
+  </si>
+  <si>
+    <t>Costco</t>
+  </si>
+  <si>
+    <t>WMT</t>
+  </si>
+  <si>
+    <t>Walmart</t>
+  </si>
+  <si>
+    <t>ORCL</t>
+  </si>
+  <si>
+    <t>Oracle</t>
+  </si>
+  <si>
+    <t>Netflix</t>
+  </si>
+  <si>
+    <t>Eli Lilly</t>
+  </si>
+  <si>
+    <t>ISRG</t>
+  </si>
+  <si>
+    <t>Intuitive Surgical</t>
+  </si>
+  <si>
+    <t>Caterpillar</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>Deere</t>
+  </si>
+  <si>
+    <t>RTX</t>
   </si>
 </sst>
 </file>
@@ -154,9 +317,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -584,12 +750,187 @@
         <v>109200</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11">
+        <v>68500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13">
+        <v>13900</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14">
+        <v>157900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15">
+        <v>12600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16">
+        <v>31900</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03B05C2C-F23D-4154-B9E7-6674A908B62A}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>407</v>
+      </c>
+      <c r="C2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>417</v>
+      </c>
+      <c r="C3">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>416</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>530</v>
+      </c>
+      <c r="C5">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>705</v>
+      </c>
+      <c r="C6">
+        <v>1165</v>
+      </c>
+      <c r="D6">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48FC485-1630-41C2-9709-BFBE7E263A58}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -671,7 +1012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{556EA6CB-4D7D-43A5-986F-1B79476B7661}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -753,7 +1094,728 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C089AC-20D9-458F-9D7D-DAF0C8478345}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>4898</v>
+      </c>
+      <c r="C2">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>4350</v>
+      </c>
+      <c r="C3">
+        <v>3049</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>4005</v>
+      </c>
+      <c r="C4">
+        <v>3086</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>4689</v>
+      </c>
+      <c r="C5">
+        <v>3174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>7943</v>
+      </c>
+      <c r="C6">
+        <v>3821</v>
+      </c>
+      <c r="D6">
+        <v>1675</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CEC2A2B-E6EE-4DEF-B916-9DCCA53D05DE}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>5.1454E-2</v>
+      </c>
+      <c r="C2">
+        <v>2.3956000000000002E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>4.9027000000000001E-2</v>
+      </c>
+      <c r="C3">
+        <v>3.3964000000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>6.6348000000000004E-2</v>
+      </c>
+      <c r="C4">
+        <v>4.1561000000000001E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>7.3640999999999998E-2</v>
+      </c>
+      <c r="C5">
+        <v>4.4548999999999998E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>7.1453000000000003E-2</v>
+      </c>
+      <c r="C6">
+        <v>3.5414000000000001E-2</v>
+      </c>
+      <c r="D6">
+        <v>3.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2156A27E-5B0C-45DE-8160-DC050F27344C}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>0.35649999999999998</v>
+      </c>
+      <c r="C2">
+        <v>0.36430000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>0.29849999999999999</v>
+      </c>
+      <c r="C3">
+        <v>0.31369999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>0.47270000000000001</v>
+      </c>
+      <c r="C4">
+        <v>0.34889999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>0.66110000000000002</v>
+      </c>
+      <c r="C5">
+        <v>0.41760000000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>0.79530000000000001</v>
+      </c>
+      <c r="C6">
+        <v>0.5071</v>
+      </c>
+      <c r="D6">
+        <v>420</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3A81782-61FA-424B-BCB9-932CF4783EAB}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>6000</v>
+      </c>
+      <c r="C2">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>7111</v>
+      </c>
+      <c r="C3">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>10234</v>
+      </c>
+      <c r="C4">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>13092</v>
+      </c>
+      <c r="C5">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>14996</v>
+      </c>
+      <c r="C6">
+        <v>594</v>
+      </c>
+      <c r="D6">
+        <v>929</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222D7682-513D-4825-BC62-A63A6B9B5A67}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>401</v>
+      </c>
+      <c r="C2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>363</v>
+      </c>
+      <c r="C3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>333</v>
+      </c>
+      <c r="C4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>700</v>
+      </c>
+      <c r="C5">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>884</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>262</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D91BFD5-CB7A-470D-B7D5-FC27A65B11E2}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2021</v>
+      </c>
+      <c r="B2">
+        <v>1135</v>
+      </c>
+      <c r="C2">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2022</v>
+      </c>
+      <c r="B3">
+        <v>1050</v>
+      </c>
+      <c r="C3">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4">
+        <v>1605</v>
+      </c>
+      <c r="C4">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
+        <v>2446</v>
+      </c>
+      <c r="C5">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>3761</v>
+      </c>
+      <c r="C6">
+        <v>1194</v>
+      </c>
+      <c r="D6">
+        <v>1200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D64AB774-227D-4BCA-8608-F74A70B0290C}">
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F6EFFA6-3D4E-40CB-9167-9611E0BB3DF4}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -802,7 +1864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C852AD-020B-43B6-920C-38E6A80F8FCC}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -896,7 +1958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C19A9A9-560B-4709-8B61-64F10DA3F3E3}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -979,7 +2041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3935994C-2385-47E7-868B-A40B19ABC727}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1061,7 +2123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B8453C4-6D6F-43DB-95E7-7C6D17636AFE}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1143,7 +2205,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44815C06-4B74-477E-90B9-68CA77F13F20}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1225,7 +2287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{211ECC06-B714-41A3-8304-4E9A77B12D43}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1299,89 +2361,7 @@
         <v>24674</v>
       </c>
       <c r="D6">
-        <v>31567</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03B05C2C-F23D-4154-B9E7-6674A908B62A}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="17.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>2021</v>
-      </c>
-      <c r="B2">
-        <v>407</v>
-      </c>
-      <c r="C2">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2022</v>
-      </c>
-      <c r="B3">
-        <v>417</v>
-      </c>
-      <c r="C3">
-        <v>922</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>2023</v>
-      </c>
-      <c r="B4">
-        <v>416</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>2024</v>
-      </c>
-      <c r="B5">
-        <v>530</v>
-      </c>
-      <c r="C5">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>2025</v>
-      </c>
-      <c r="B6">
-        <v>705</v>
-      </c>
-      <c r="C6">
-        <v>1165</v>
-      </c>
-      <c r="D6">
-        <v>85</v>
+        <v>31.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>